<commit_message>
perf(Layer): BSP层提供初始化Hardware Source Register接口。
</commit_message>
<xml_diff>
--- a/OV_F407VGT6_2026.01.18/天空星引脚配置.xlsx
+++ b/OV_F407VGT6_2026.01.18/天空星引脚配置.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\振动式粘度计\01_Project_Management\OV_F407VGT6_2026.01.18\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Oscillatory_Viscometer\01_Project_Management\OV_F407VGT6_2026.01.18\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C3FB99-5AF1-48B6-AF5E-1B5EBD086EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A11A42A3-F064-477C-BA65-A5D0D1CEF9DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -418,15 +418,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>6.045kSPS（0x00A2）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>3.008kSPS（0x0149）</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>斥力驱动</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6.045kSPS（0x00A3）</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1945,10 +1945,10 @@
         <v>197</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
@@ -1971,7 +1971,7 @@
         <v>89</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -1990,11 +1990,11 @@
         <v>1000</v>
       </c>
       <c r="H28" s="1">
-        <v>269</v>
+        <v>1046</v>
       </c>
       <c r="I28" s="39"/>
       <c r="J28" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="I29" s="39"/>
       <c r="J29" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>